<commit_message>
Reorder days 5-7: move Bayeux+Omaha+Etretat before Mont-Saint-Michel, update HTML, Excel and KML accordingly.
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/v3/itinerary.xlsx
+++ b/v3/itinerary.xlsx
@@ -1201,30 +1201,90 @@
       </c>
       <c r="D9" s="21" t="inlineStr">
         <is>
-          <t>→ Mont-Saint-Michel</t>
+          <t>Bayeux + Omaha + Etretat</t>
         </is>
       </c>
       <c r="E9" s="22" t="inlineStr">
         <is>
-          <t>~380 km</t>
+          <t>~260 km</t>
         </is>
       </c>
       <c r="F9" s="23" t="inlineStr">
         <is>
-          <t>Giornata di trasferimento. Partenza presto (ore 7:00). A11 → Le Mans (sosta 30 min facoltativa, Vieille Ville con mura romane) → N157 → Mont-Saint-Michel. ~4h di guida.</t>
+          <t>Giornata di trasferimento + visita. Partenza ore 7:00. A13 direzione Caen -&gt; Bayeux (~2h30). Bayeux (9:00): Arazzo XI sec. (70m di storia normanna, 1h), cattedrale. Omaha Beach + Cimitero Americano di Colleville-sur-Mer. Pointe du Hoc: trincee e crateri intatti. Pranzo a Port-en-Bessin (porto peschereccio).</t>
         </is>
       </c>
       <c r="G9" s="23" t="inlineStr">
         <is>
-          <t>⚠ ARRIVARE DOPO LE 17 — luce magica sull'abbazia, folla ridotta. Parcheggio camper parking continentale (prenotare su visite-mont-saint-michel.com). Navette gratuite. Prima impressione al tramonto.</t>
+          <t>Etretat (15:00): scogliere bianche piu famose d'Europa, passeggiata sulle falaise (1h, facile). Tramonto spettacolare da lassu.</t>
         </is>
       </c>
       <c r="H9" s="23" t="inlineStr">
         <is>
+          <t>Camping Municipal d'Étretat ★★★ (prato dietro le scogliere)</t>
+        </is>
+      </c>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>1. Camping Port'land — Port-en-Bessin ★★★★★
+   Sul porto, piscina coperta
+2. Camping de Bayeux ★★★★
+   In città, 800m dall'Arazzo
+3. Camping La Chêneraie — Fécamp ★★★★
+   20 km da Étretat, più tranquillo</t>
+        </is>
+      </c>
+      <c r="J9" s="23" t="inlineStr">
+        <is>
+          <t>1. Aire de Bayeux
+   SC · AC · EL · WC | 500m Arazzo
+2. Aire de Port-en-Bessin
+   SC · AC · WC | Sul porto, gratuita
+3. Aire d'Étretat
+   SC · AC · WC | 200m scogliere</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90" customHeight="1">
+      <c r="A10" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>Mer 26 ago</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>Normandia</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>-&gt; Mont-Saint-Michel</t>
+        </is>
+      </c>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>~190 km</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="inlineStr">
+        <is>
+          <t>Giornata di trasferimento. Partenza ore 7:00. D925 -&gt; Honfleur (sosta caffe facoltativa) -&gt; A29 -&gt; Caen -&gt; A84 -&gt; Mont-Saint-Michel. ~2h30 di guida.</t>
+        </is>
+      </c>
+      <c r="G10" s="23" t="inlineStr">
+        <is>
+          <t>ARRIVARE DOPO LE 17 - luce magica sull'abbazia, folla ridotta. Parcheggio camper parking continentale (prenotare su visite-mont-saint-michel.com). Navette gratuite. Prima impressione al tramonto.</t>
+        </is>
+      </c>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
           <t>Camping Haliotis — Pontorson ★★★★ (8 km, navetta inclusa) — PRENOTARE</t>
         </is>
       </c>
-      <c r="I9" s="23" t="inlineStr">
+      <c r="I10" s="23" t="inlineStr">
         <is>
           <t>1. Camping du Mont-Saint-Michel ★★★★
    Il più vicino (2 km), vista abbazia
@@ -1234,7 +1294,7 @@
    9 km, tranquillo, prezzi accessibili</t>
         </is>
       </c>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>1. Aire Officielle Mont-Saint-Michel — Beauvoir
    SC · AC · EL · WC · DU | Ufficiale, navetta. PRENOTARE
@@ -1245,46 +1305,46 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="19" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="20" t="inlineStr">
-        <is>
-          <t>Mer 26 ago</t>
-        </is>
-      </c>
-      <c r="C10" s="20" t="inlineStr">
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>Gio 27 ago</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>Normandia</t>
         </is>
       </c>
-      <c r="D10" s="21" t="inlineStr">
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>Mont-Saint-Michel + costa</t>
         </is>
       </c>
-      <c r="E10" s="22" t="inlineStr">
+      <c r="E11" s="22" t="inlineStr">
         <is>
           <t>~80 km</t>
         </is>
       </c>
-      <c r="F10" s="23" t="inlineStr">
+      <c r="F11" s="23" t="inlineStr">
         <is>
           <t>Mont-Saint-Michel (9:00–12:00): abbazia benedettina, borgo medievale, camminata sulle mura. Verificare orari maree — tra le più forti d'Europa. Salita impegnativa ma i bambini reggono bene.</t>
         </is>
       </c>
-      <c r="G10" s="23" t="inlineStr">
+      <c r="G11" s="23" t="inlineStr">
         <is>
           <t>Pomeriggio: spiagge tranquille della Côte des Havres — sabbiose, poco frequentate, perfette per i bambini dopo giorni intensi. Sera a Granville o Avranches: pesce fresco.</t>
         </is>
       </c>
-      <c r="H10" s="23" t="inlineStr">
+      <c r="H11" s="23" t="inlineStr">
         <is>
           <t>Camping La Vague — Jullouville ★★★★ (direttamente sul mare)</t>
         </is>
       </c>
-      <c r="I10" s="23" t="inlineStr">
+      <c r="I11" s="23" t="inlineStr">
         <is>
           <t>1. Camping du Mont-Saint-Michel ★★★★
    Restare vicino al sito
@@ -1294,7 +1354,7 @@
    Spiaggia a 200m</t>
         </is>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>1. Aire de Pontorson
    SC · AC · WC | Gratuita, 8 km Mont
@@ -1302,66 +1362,6 @@
    SC · AC · EL · WC | Vista mare
 3. Aire de Avranches
    SC · AC · WC | In città</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="90" customHeight="1">
-      <c r="A11" s="19" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="20" t="inlineStr">
-        <is>
-          <t>Gio 27 ago</t>
-        </is>
-      </c>
-      <c r="C11" s="20" t="inlineStr">
-        <is>
-          <t>Normandia</t>
-        </is>
-      </c>
-      <c r="D11" s="21" t="inlineStr">
-        <is>
-          <t>Bayeux + Omaha + Étretat</t>
-        </is>
-      </c>
-      <c r="E11" s="22" t="inlineStr">
-        <is>
-          <t>~130 km</t>
-        </is>
-      </c>
-      <c r="F11" s="23" t="inlineStr">
-        <is>
-          <t>Bayeux (9:00): Arazzo XI sec. (70m di storia normanna, 1h), cattedrale. Omaha Beach + Cimitero Americano di Colleville-sur-Mer — luogo di grande impatto emotivo. Pointe du Hoc: trincee e crateri intatti. Pranzo a Port-en-Bessin (porto peschereccio).</t>
-        </is>
-      </c>
-      <c r="G11" s="23" t="inlineStr">
-        <is>
-          <t>Étretat (15:00): scogliere bianche più famose d'Europa, passeggiata sulle falaise (1h, facile). Tramonto spettacolare da lassù.</t>
-        </is>
-      </c>
-      <c r="H11" s="23" t="inlineStr">
-        <is>
-          <t>Camping Municipal d'Étretat ★★★ (prato dietro le scogliere)</t>
-        </is>
-      </c>
-      <c r="I11" s="23" t="inlineStr">
-        <is>
-          <t>1. Camping Port'land — Port-en-Bessin ★★★★★
-   Sul porto, piscina coperta
-2. Camping de Bayeux ★★★★
-   In città, 800m dall'Arazzo
-3. Camping La Chêneraie — Fécamp ★★★★
-   20 km da Étretat, più tranquillo</t>
-        </is>
-      </c>
-      <c r="J11" s="23" t="inlineStr">
-        <is>
-          <t>1. Aire de Bayeux
-   SC · AC · EL · WC | 500m Arazzo
-2. Aire de Port-en-Bessin
-   SC · AC · WC | Sul porto, gratuita
-3. Aire d'Étretat
-   SC · AC · WC | 200m scogliere</t>
         </is>
       </c>
     </row>

</xml_diff>